<commit_message>
docs: sincronizar carpeta Listo desde main
</commit_message>
<xml_diff>
--- a/Fase_2/Evidencias Proyecto/Evidencias de documentación/Listo/EDT_SIGFQ.xlsx
+++ b/Fase_2/Evidencias Proyecto/Evidencias de documentación/Listo/EDT_SIGFQ.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alvar\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alvar\Documents\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A55F3918-130E-4D61-B7BE-4B8FD22FEDAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDFF8A7E-F772-4787-AB73-3ADCC3AE2D2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -761,6 +761,32 @@
     <xf numFmtId="1" fontId="16" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -787,32 +813,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1475,16 +1475,16 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="37.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="55" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="47"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="57"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -1536,20 +1536,20 @@
         <v>0</v>
       </c>
       <c r="B4" s="12"/>
-      <c r="C4" s="48" t="s">
+      <c r="C4" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
-      <c r="H4" s="50"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="59"/>
+      <c r="F4" s="59"/>
+      <c r="G4" s="59"/>
+      <c r="H4" s="60"/>
       <c r="I4" s="9"/>
-      <c r="J4" s="51" t="s">
+      <c r="J4" s="61" t="s">
         <v>2</v>
       </c>
-      <c r="K4" s="49"/>
-      <c r="L4" s="50"/>
+      <c r="K4" s="59"/>
+      <c r="L4" s="60"/>
       <c r="M4" s="9"/>
       <c r="N4" s="9"/>
       <c r="O4" s="9"/>
@@ -1641,7 +1641,7 @@
       <c r="K6" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="L6" s="65" t="s">
+      <c r="L6" s="53" t="s">
         <v>101</v>
       </c>
       <c r="M6" s="20">
@@ -1682,7 +1682,7 @@
       <c r="K7" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="L7" s="65" t="s">
+      <c r="L7" s="53" t="s">
         <v>100</v>
       </c>
       <c r="M7" s="22">
@@ -1725,7 +1725,7 @@
       <c r="K8" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="L8" s="65" t="s">
+      <c r="L8" s="53" t="s">
         <v>102</v>
       </c>
       <c r="M8" s="22">
@@ -2085,10 +2085,10 @@
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
-      <c r="L17" s="52" t="s">
+      <c r="L17" s="62" t="s">
         <v>22</v>
       </c>
-      <c r="M17" s="50"/>
+      <c r="M17" s="60"/>
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
       <c r="P17" s="1"/>
@@ -2104,16 +2104,16 @@
       <c r="Z17" s="1"/>
     </row>
     <row r="18" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="59" t="s">
+      <c r="A18" s="47" t="s">
         <v>66</v>
       </c>
-      <c r="B18" s="60"/>
-      <c r="C18" s="61"/>
-      <c r="D18" s="61"/>
-      <c r="E18" s="61"/>
-      <c r="F18" s="61"/>
-      <c r="G18" s="61"/>
-      <c r="H18" s="61"/>
+      <c r="B18" s="48"/>
+      <c r="C18" s="49"/>
+      <c r="D18" s="49"/>
+      <c r="E18" s="49"/>
+      <c r="F18" s="49"/>
+      <c r="G18" s="49"/>
+      <c r="H18" s="49"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
@@ -2143,7 +2143,7 @@
         <v>67</v>
       </c>
       <c r="B19" s="21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C19" s="18"/>
       <c r="D19" s="18">
@@ -2184,7 +2184,7 @@
         <v>68</v>
       </c>
       <c r="B20" s="21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C20" s="18"/>
       <c r="D20" s="18"/>
@@ -2223,7 +2223,7 @@
         <v>69</v>
       </c>
       <c r="B21" s="21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C21" s="18">
         <v>3</v>
@@ -2262,16 +2262,16 @@
       <c r="Z21" s="1"/>
     </row>
     <row r="22" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="57" t="s">
+      <c r="A22" s="45" t="s">
         <v>71</v>
       </c>
-      <c r="B22" s="62"/>
-      <c r="C22" s="58"/>
-      <c r="D22" s="58"/>
-      <c r="E22" s="58"/>
-      <c r="F22" s="58"/>
-      <c r="G22" s="58"/>
-      <c r="H22" s="58"/>
+      <c r="B22" s="50"/>
+      <c r="C22" s="46"/>
+      <c r="D22" s="46"/>
+      <c r="E22" s="46"/>
+      <c r="F22" s="46"/>
+      <c r="G22" s="46"/>
+      <c r="H22" s="46"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
@@ -2350,10 +2350,10 @@
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
-      <c r="L24" s="52" t="s">
+      <c r="L24" s="62" t="s">
         <v>24</v>
       </c>
-      <c r="M24" s="50"/>
+      <c r="M24" s="60"/>
       <c r="N24" s="1"/>
       <c r="O24" s="1"/>
       <c r="P24" s="1"/>
@@ -2412,16 +2412,16 @@
       <c r="Z25" s="1"/>
     </row>
     <row r="26" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="63" t="s">
+      <c r="A26" s="51" t="s">
         <v>76</v>
       </c>
-      <c r="B26" s="64"/>
-      <c r="C26" s="64"/>
-      <c r="D26" s="64"/>
-      <c r="E26" s="64"/>
-      <c r="F26" s="64"/>
-      <c r="G26" s="64"/>
-      <c r="H26" s="64"/>
+      <c r="B26" s="52"/>
+      <c r="C26" s="52"/>
+      <c r="D26" s="52"/>
+      <c r="E26" s="52"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="52"/>
+      <c r="H26" s="52"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
@@ -2607,16 +2607,16 @@
       <c r="Z30" s="1"/>
     </row>
     <row r="31" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="63" t="s">
+      <c r="A31" s="51" t="s">
         <v>80</v>
       </c>
-      <c r="B31" s="64"/>
-      <c r="C31" s="64"/>
-      <c r="D31" s="64"/>
-      <c r="E31" s="64"/>
-      <c r="F31" s="64"/>
-      <c r="G31" s="64"/>
-      <c r="H31" s="64"/>
+      <c r="B31" s="52"/>
+      <c r="C31" s="52"/>
+      <c r="D31" s="52"/>
+      <c r="E31" s="52"/>
+      <c r="F31" s="52"/>
+      <c r="G31" s="52"/>
+      <c r="H31" s="52"/>
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
@@ -2757,16 +2757,16 @@
       <c r="Z34" s="1"/>
     </row>
     <row r="35" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="63" t="s">
+      <c r="A35" s="51" t="s">
         <v>86</v>
       </c>
-      <c r="B35" s="64"/>
-      <c r="C35" s="64"/>
-      <c r="D35" s="64"/>
-      <c r="E35" s="64"/>
-      <c r="F35" s="64"/>
-      <c r="G35" s="64"/>
-      <c r="H35" s="64"/>
+      <c r="B35" s="52"/>
+      <c r="C35" s="52"/>
+      <c r="D35" s="52"/>
+      <c r="E35" s="52"/>
+      <c r="F35" s="52"/>
+      <c r="G35" s="52"/>
+      <c r="H35" s="52"/>
       <c r="I35" s="1"/>
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
@@ -3242,7 +3242,7 @@
       <c r="Z47" s="1"/>
     </row>
     <row r="48" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="66" t="s">
+      <c r="A48" s="54" t="s">
         <v>103</v>
       </c>
       <c r="B48" s="21">
@@ -29911,29 +29911,29 @@
   <sheetData>
     <row r="1" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H2" s="53" t="s">
+      <c r="H2" s="63" t="s">
         <v>32</v>
       </c>
-      <c r="I2" s="54"/>
-      <c r="J2" s="54"/>
-      <c r="K2" s="54"/>
-      <c r="L2" s="54"/>
-      <c r="M2" s="54"/>
+      <c r="I2" s="64"/>
+      <c r="J2" s="64"/>
+      <c r="K2" s="64"/>
+      <c r="L2" s="64"/>
+      <c r="M2" s="64"/>
     </row>
     <row r="3" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H3" s="55" t="s">
+      <c r="H3" s="65" t="s">
         <v>33</v>
       </c>
-      <c r="I3" s="54"/>
-      <c r="J3" s="54"/>
-      <c r="K3" s="54"/>
+      <c r="I3" s="64"/>
+      <c r="J3" s="64"/>
+      <c r="K3" s="64"/>
     </row>
     <row r="4" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C4" s="56" t="s">
+      <c r="C4" s="66" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="49"/>
-      <c r="E4" s="50"/>
+      <c r="D4" s="59"/>
+      <c r="E4" s="60"/>
     </row>
     <row r="5" spans="1:13" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
@@ -30164,12 +30164,12 @@
     <row r="21" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="22" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="23" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="H23" s="55" t="s">
+      <c r="H23" s="65" t="s">
         <v>53</v>
       </c>
-      <c r="I23" s="54"/>
-      <c r="J23" s="54"/>
-      <c r="K23" s="54"/>
+      <c r="I23" s="64"/>
+      <c r="J23" s="64"/>
+      <c r="K23" s="64"/>
     </row>
     <row r="24" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="25" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -30190,12 +30190,12 @@
     <row r="40" spans="8:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="41" spans="8:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="42" spans="8:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H42" s="53" t="s">
+      <c r="H42" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="I42" s="54"/>
-      <c r="J42" s="54"/>
-      <c r="K42" s="54"/>
+      <c r="I42" s="64"/>
+      <c r="J42" s="64"/>
+      <c r="K42" s="64"/>
     </row>
     <row r="43" spans="8:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="44" spans="8:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>